<commit_message>
chore: snapshot current RPA integration state for full audit
</commit_message>
<xml_diff>
--- a/outlook-rpa-dashboard/api/generated/checklists/VARIETYWHO/1885387-CHECKLIST.xlsx
+++ b/outlook-rpa-dashboard/api/generated/checklists/VARIETYWHO/1885387-CHECKLIST.xlsx
@@ -1578,12 +1578,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns5="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D254"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75" ns3:dyDescent="0.2"/>
+  <dimension ref="A1:H254"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="39.140625" customWidth="1"/>
     <col min="2" max="2" width="21.140625" customWidth="1"/>
@@ -1596,35 +1596,39 @@
     <col min="10" max="10" width="11.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="33" customHeight="1" thickBot="1" ns3:dyDescent="0.45">
+    <row r="1" spans="1:8" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B1" s="61" t="s">
         <v>29</v>
       </c>
       <c r="C1" s="62"/>
       <c r="D1" s="63"/>
     </row>
-    <row r="3" spans="1:8" ht="21" customHeight="1" ns3:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="39" t="s">
-        <v>33</v>
+      <c r="C3" s="39" t="inlineStr">
+        <is>
+          <t>PT#</t>
+        </is>
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="12"/>
     </row>
-    <row r="4" spans="1:8" ht="15" ns3:dyDescent="0.2">
-      <c r="C4" s="39" t="s">
-        <v>34</v>
+    <row r="4" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="C4" s="39" t="inlineStr">
+        <is>
+          <t>PO# 1885387</t>
+        </is>
       </c>
       <c r="D4" s="12"/>
       <c r="F4" s="12"/>
     </row>
-    <row r="5" spans="1:8" ht="14.25" customHeight="1" ns3:dyDescent="0.2">
+    <row r="5" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="E5" s="12"/>
       <c r="F5" s="12"/>
     </row>
-    <row r="6" spans="1:8" ht="127.5" ns3:dyDescent="0.2">
+    <row r="6" spans="1:8" ht="127.5" x14ac:dyDescent="0.2">
       <c r="A6" s="24" t="s">
         <v>1</v>
       </c>
@@ -1639,19 +1643,19 @@
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
     </row>
-    <row r="7" spans="1:8" ns3:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="23"/>
       <c r="D7" s="37"/>
       <c r="E7" s="31"/>
       <c r="F7" s="12"/>
     </row>
-    <row r="8" spans="1:8" ns3:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="23"/>
       <c r="D8" s="38"/>
       <c r="E8" s="31"/>
       <c r="F8" s="12"/>
     </row>
-    <row r="9" spans="1:8" ns3:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="24" t="s">
         <v>2</v>
       </c>
@@ -1662,20 +1666,20 @@
       <c r="E9" s="30"/>
       <c r="F9" s="12"/>
     </row>
-    <row r="10" spans="1:8" ht="12.75" customHeight="1" ns3:dyDescent="0.2">
+    <row r="10" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="E10" s="12"/>
       <c r="F10" s="12"/>
     </row>
-    <row r="11" spans="1:8" ns3:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E11" s="12"/>
       <c r="F11" s="12"/>
     </row>
-    <row r="12" spans="1:8" ht="13.5" thickBot="1" ns3:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D12" s="20"/>
       <c r="E12" s="12"/>
       <c r="F12" s="12"/>
     </row>
-    <row r="13" spans="1:8" ht="35.25" customHeight="1" thickBot="1" ns3:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="35.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="28" t="s">
         <v>3</v>
       </c>
@@ -1686,7 +1690,7 @@
       <c r="D13" s="60"/>
       <c r="E13" s="12"/>
     </row>
-    <row r="14" spans="1:8" ht="38.25" ns3:dyDescent="0.2">
+    <row r="14" spans="1:8" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A14" s="64" t="s">
         <v>11</v>
       </c>
@@ -1699,7 +1703,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ns3:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>4</v>
       </c>
@@ -1710,7 +1714,7 @@
       <c r="D15" s="18"/>
       <c r="E15" s="12"/>
     </row>
-    <row r="16" spans="1:8" ht="15" ns3:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>5</v>
       </c>
@@ -1721,7 +1725,7 @@
       <c r="D16" s="18"/>
       <c r="E16" s="12"/>
     </row>
-    <row r="17" spans="1:7" ht="15" ns3:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>22</v>
       </c>
@@ -1740,7 +1744,7 @@
       </c>
       <c r="E17" s="12"/>
     </row>
-    <row r="18" spans="1:7" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>21</v>
       </c>
@@ -1755,7 +1759,7 @@
       </c>
       <c r="E18" s="12"/>
     </row>
-    <row r="19" spans="1:7" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>16</v>
       </c>
@@ -1766,7 +1770,7 @@
       <c r="D19" s="18"/>
       <c r="E19" s="12"/>
     </row>
-    <row r="20" spans="1:7" ht="15" ns3:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>10</v>
       </c>
@@ -1777,7 +1781,7 @@
       <c r="D20" s="18"/>
       <c r="E20" s="12"/>
     </row>
-    <row r="21" spans="1:7" ns3:dyDescent="0.2">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
         <v>27</v>
       </c>
@@ -1789,7 +1793,7 @@
       <c r="E21" s="12"/>
       <c r="F21" s="13"/>
     </row>
-    <row r="22" spans="1:7" ht="15.75" thickBot="1" ns3:dyDescent="0.3">
+    <row r="22" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
         <v>19</v>
       </c>
@@ -1800,7 +1804,7 @@
       <c r="D22" s="19"/>
       <c r="E22" s="12"/>
     </row>
-    <row r="23" spans="1:7" ht="12.75" customHeight="1" ns3:dyDescent="0.2">
+    <row r="23" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="57" t="s">
         <v>17</v>
       </c>
@@ -1810,7 +1814,7 @@
       <c r="E23" s="12"/>
       <c r="F23" s="12"/>
     </row>
-    <row r="24" spans="1:7" ht="24" customHeight="1" ns3:dyDescent="0.2">
+    <row r="24" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="58"/>
       <c r="B24" s="58"/>
       <c r="C24" s="58"/>
@@ -1818,7 +1822,7 @@
       <c r="E24" s="12"/>
       <c r="F24" s="12"/>
     </row>
-    <row r="25" spans="1:7" ns3:dyDescent="0.2">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" s="11" t="s">
         <v>6</v>
       </c>
@@ -1841,7 +1845,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:7" s="49" customFormat="1" ht="15" ns3:dyDescent="0.25">
+    <row r="26" spans="1:7" s="49" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A26" s="53" t="inlineStr">
         <is>
           <t>W7EH00709-42</t>
@@ -1868,7 +1872,7 @@
       <c r="F26" s="50"/>
       <c r="G26" s="51"/>
     </row>
-    <row r="27" spans="1:7" s="49" customFormat="1" ht="15" ns3:dyDescent="0.25">
+    <row r="27" spans="1:7" s="49" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A27" s="53" t="inlineStr">
         <is>
           <t>W7EH00184-42</t>
@@ -1895,7 +1899,7 @@
       <c r="F27" s="52"/>
       <c r="G27" s="51"/>
     </row>
-    <row r="28" spans="1:7" s="73" customFormat="1" ht="15" ns3:dyDescent="0.25">
+    <row r="28" spans="1:7" s="73" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A28" s="66" t="inlineStr">
         <is>
           <t>W7EH1122-42</t>
@@ -1922,7 +1926,7 @@
       <c r="F28" s="72"/>
       <c r="G28" s="70"/>
     </row>
-    <row r="29" spans="1:7" s="49" customFormat="1" ht="15" ns3:dyDescent="0.25">
+    <row r="29" spans="1:7" s="49" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A29" s="53" t="inlineStr">
         <is>
           <t>W7EH00081-42</t>
@@ -1949,7 +1953,7 @@
       <c r="F29" s="52"/>
       <c r="G29" s="51"/>
     </row>
-    <row r="30" spans="1:7" s="71" customFormat="1" ht="15" ns3:dyDescent="0.25">
+    <row r="30" spans="1:7" s="71" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A30" s="66" t="inlineStr">
         <is>
           <t>W7EH00713-42</t>
@@ -1976,7 +1980,7 @@
       <c r="F30" s="69"/>
       <c r="G30" s="70"/>
     </row>
-    <row r="31" spans="1:7" ht="15" ns3:dyDescent="0.25">
+    <row r="31" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A31" s="53" t="inlineStr">
         <is>
           <t>W7EH1123-42</t>
@@ -2003,7 +2007,7 @@
       <c r="F31" s="50"/>
       <c r="G31" s="51"/>
     </row>
-    <row r="32" spans="1:7" ht="15" ns3:dyDescent="0.25">
+    <row r="32" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A32" s="53" t="inlineStr">
         <is>
           <t>W7AB00176-42</t>
@@ -2030,7 +2034,7 @@
       <c r="F32" s="50"/>
       <c r="G32" s="51"/>
     </row>
-    <row r="33" spans="1:7" ht="15" ns3:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A33" s="53" t="inlineStr">
         <is>
           <t>W7AB1149-42</t>
@@ -2057,7 +2061,7 @@
       <c r="F33" s="50"/>
       <c r="G33" s="51"/>
     </row>
-    <row r="34" spans="1:7" ht="15" ns3:dyDescent="0.25">
+    <row r="34" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A34" s="53" t="inlineStr">
         <is>
           <t>W7AB00174-42</t>
@@ -2084,227 +2088,128 @@
       <c r="F34" s="50"/>
       <c r="G34" s="51"/>
     </row>
-    <row r="35" spans="1:7" ht="15" ns3:dyDescent="0.25">
-      <c r="A35" s="53" t="s">
-        <v>40</v>
-      </c>
-      <c r="B35" s="53" t="s">
-        <v>50</v>
-      </c>
-      <c r="C35" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v>W5EH00521-42-009</v>
-      </c>
-      <c r="D35" s="55">
-        <v>298201</v>
-      </c>
+    <row r="35" spans="1:7" ht="15" x14ac:dyDescent="0.25" hidden="1">
+      <c r="A35" s="53"/>
+      <c r="B35" s="53"/>
+      <c r="C35" s="54"/>
+      <c r="D35" s="55"/>
       <c r="E35" s="53">
         <v>96</v>
       </c>
       <c r="F35" s="50"/>
       <c r="G35" s="51"/>
     </row>
-    <row r="36" spans="1:7" ht="15" ns3:dyDescent="0.25">
-      <c r="A36" s="53" t="s">
-        <v>41</v>
-      </c>
-      <c r="B36" s="53" t="s">
-        <v>46</v>
-      </c>
-      <c r="C36" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v>W5EH00863-42-033</v>
-      </c>
-      <c r="D36" s="55">
-        <v>298204</v>
-      </c>
+    <row r="36" spans="1:7" ht="15" x14ac:dyDescent="0.25" hidden="1">
+      <c r="A36" s="53"/>
+      <c r="B36" s="53"/>
+      <c r="C36" s="54"/>
+      <c r="D36" s="55"/>
       <c r="E36" s="53">
         <v>144</v>
       </c>
       <c r="F36" s="50"/>
       <c r="G36" s="51"/>
     </row>
-    <row r="37" spans="1:7" ht="15" ns3:dyDescent="0.25">
-      <c r="A37" s="53" t="s">
-        <v>41</v>
-      </c>
-      <c r="B37" s="53" t="s">
-        <v>46</v>
-      </c>
-      <c r="C37" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v>W5EH00863-42-033</v>
-      </c>
-      <c r="D37" s="55">
-        <v>298204</v>
-      </c>
+    <row r="37" spans="1:7" ht="15" x14ac:dyDescent="0.25" hidden="1">
+      <c r="A37" s="53"/>
+      <c r="B37" s="53"/>
+      <c r="C37" s="54"/>
+      <c r="D37" s="55"/>
       <c r="E37" s="53">
         <v>96</v>
       </c>
       <c r="F37" s="56"/>
       <c r="G37" s="56"/>
     </row>
-    <row r="38" spans="1:7" ht="15" ns3:dyDescent="0.25">
-      <c r="A38" s="53" t="s">
-        <v>42</v>
-      </c>
-      <c r="B38" s="53" t="s">
-        <v>49</v>
-      </c>
-      <c r="C38" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v>W5EH00864-42-003</v>
-      </c>
-      <c r="D38" s="55">
-        <v>298202</v>
-      </c>
+    <row r="38" spans="1:7" ht="15" x14ac:dyDescent="0.25" hidden="1">
+      <c r="A38" s="53"/>
+      <c r="B38" s="53"/>
+      <c r="C38" s="54"/>
+      <c r="D38" s="55"/>
       <c r="E38" s="53">
         <v>144</v>
       </c>
       <c r="F38" s="50"/>
       <c r="G38" s="51"/>
     </row>
-    <row r="39" spans="1:7" ht="15" ns3:dyDescent="0.25">
-      <c r="A39" s="53" t="s">
-        <v>42</v>
-      </c>
-      <c r="B39" s="53" t="s">
-        <v>49</v>
-      </c>
-      <c r="C39" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v>W5EH00864-42-003</v>
-      </c>
-      <c r="D39" s="55">
-        <v>298202</v>
-      </c>
+    <row r="39" spans="1:7" ht="15" x14ac:dyDescent="0.25" hidden="1">
+      <c r="A39" s="53"/>
+      <c r="B39" s="53"/>
+      <c r="C39" s="54"/>
+      <c r="D39" s="55"/>
       <c r="E39" s="53">
         <v>96</v>
       </c>
       <c r="F39" s="50"/>
       <c r="G39" s="51"/>
     </row>
-    <row r="40" spans="1:7" s="71" customFormat="1" ht="15" ns3:dyDescent="0.25">
-      <c r="A40" s="66" t="s">
-        <v>43</v>
-      </c>
-      <c r="B40" s="66" t="s">
-        <v>47</v>
-      </c>
-      <c r="C40" s="67" t="str">
-        <f t="shared" si="0"/>
-        <v>W8OK1283-42-010</v>
-      </c>
-      <c r="D40" s="55">
-        <v>298225</v>
-      </c>
+    <row r="40" spans="1:7" s="71" customFormat="1" ht="15" x14ac:dyDescent="0.25" hidden="1">
+      <c r="A40" s="66"/>
+      <c r="B40" s="66"/>
+      <c r="C40" s="67"/>
+      <c r="D40" s="55"/>
       <c r="E40" s="66">
         <v>96</v>
       </c>
       <c r="F40" s="69"/>
       <c r="G40" s="70"/>
     </row>
-    <row r="41" spans="1:7" ht="15" ns3:dyDescent="0.25">
-      <c r="A41" s="53" t="s">
-        <v>43</v>
-      </c>
-      <c r="B41" s="53" t="s">
-        <v>47</v>
-      </c>
-      <c r="C41" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v>W8OK1283-42-010</v>
-      </c>
-      <c r="D41" s="55">
-        <v>298225</v>
-      </c>
+    <row r="41" spans="1:7" ht="15" x14ac:dyDescent="0.25" hidden="1">
+      <c r="A41" s="53"/>
+      <c r="B41" s="53"/>
+      <c r="C41" s="54"/>
+      <c r="D41" s="55"/>
       <c r="E41" s="53">
         <v>96</v>
       </c>
       <c r="F41" s="50"/>
       <c r="G41" s="51"/>
     </row>
-    <row r="42" spans="1:7" ht="15" ns3:dyDescent="0.25">
-      <c r="A42" s="45" t="s">
-        <v>44</v>
-      </c>
-      <c r="B42" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="C42" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v>W8OK1289-42-BCT</v>
-      </c>
-      <c r="D42" s="55">
-        <v>298226</v>
-      </c>
+    <row r="42" spans="1:7" ht="15" x14ac:dyDescent="0.25" hidden="1">
+      <c r="A42" s="45"/>
+      <c r="B42" s="45"/>
+      <c r="C42" s="54"/>
+      <c r="D42" s="55"/>
       <c r="E42" s="45">
         <v>96</v>
       </c>
       <c r="F42" s="36"/>
       <c r="G42" s="35"/>
     </row>
-    <row r="43" spans="1:7" ht="15" ns3:dyDescent="0.25">
-      <c r="A43" s="45" t="s">
-        <v>44</v>
-      </c>
-      <c r="B43" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="C43" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v>W8OK1289-42-BCT</v>
-      </c>
-      <c r="D43" s="55">
-        <v>298226</v>
-      </c>
+    <row r="43" spans="1:7" ht="15" x14ac:dyDescent="0.25" hidden="1">
+      <c r="A43" s="45"/>
+      <c r="B43" s="45"/>
+      <c r="C43" s="54"/>
+      <c r="D43" s="55"/>
       <c r="E43" s="45">
         <v>96</v>
       </c>
       <c r="F43" s="36"/>
       <c r="G43" s="35"/>
     </row>
-    <row r="44" spans="1:7" ht="15" ns3:dyDescent="0.25">
-      <c r="A44" s="45" t="s">
-        <v>45</v>
-      </c>
-      <c r="B44" s="45" t="s">
-        <v>52</v>
-      </c>
-      <c r="C44" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v>W8WM1280-42-OSD</v>
-      </c>
-      <c r="D44" s="55">
-        <v>298227</v>
-      </c>
+    <row r="44" spans="1:7" ht="15" x14ac:dyDescent="0.25" hidden="1">
+      <c r="A44" s="45"/>
+      <c r="B44" s="45"/>
+      <c r="C44" s="54"/>
+      <c r="D44" s="55"/>
       <c r="E44" s="45">
         <v>96</v>
       </c>
       <c r="F44" s="36"/>
       <c r="G44" s="35"/>
     </row>
-    <row r="45" spans="1:7" ht="15" ns3:dyDescent="0.25">
-      <c r="A45" s="45" t="s">
-        <v>45</v>
-      </c>
-      <c r="B45" s="45" t="s">
-        <v>52</v>
-      </c>
-      <c r="C45" s="54" t="str">
-        <f t="shared" si="0"/>
-        <v>W8WM1280-42-OSD</v>
-      </c>
-      <c r="D45" s="55">
-        <v>298227</v>
-      </c>
+    <row r="45" spans="1:7" ht="15" x14ac:dyDescent="0.25" hidden="1">
+      <c r="A45" s="45"/>
+      <c r="B45" s="45"/>
+      <c r="C45" s="54"/>
+      <c r="D45" s="55"/>
       <c r="E45" s="45">
         <v>96</v>
       </c>
       <c r="F45" s="36"/>
       <c r="G45" s="35"/>
     </row>
-    <row r="46" spans="1:7" ns3:dyDescent="0.2">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" s="45"/>
       <c r="B46" s="45"/>
       <c r="C46" s="35"/>
@@ -2313,7 +2218,7 @@
       <c r="F46" s="36"/>
       <c r="G46" s="35"/>
     </row>
-    <row r="47" spans="1:7" ns3:dyDescent="0.2">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" s="45"/>
       <c r="B47" s="45"/>
       <c r="C47" s="35"/>
@@ -2322,7 +2227,7 @@
       <c r="F47" s="36"/>
       <c r="G47" s="35"/>
     </row>
-    <row r="48" spans="1:7" ns3:dyDescent="0.2">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48" s="45"/>
       <c r="B48" s="45"/>
       <c r="C48" s="35"/>
@@ -2331,14 +2236,14 @@
       <c r="F48" s="36"/>
       <c r="G48" s="35"/>
     </row>
-    <row r="49" spans="1:7" ns3:dyDescent="0.2">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C49" s="44"/>
       <c r="D49" s="44"/>
       <c r="E49" s="48"/>
       <c r="F49" s="47"/>
       <c r="G49" s="44"/>
     </row>
-    <row r="50" spans="1:7" ns3:dyDescent="0.2">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" s="33"/>
       <c r="B50" s="33"/>
       <c r="C50" s="33"/>
@@ -2347,7 +2252,7 @@
       <c r="F50" s="36"/>
       <c r="G50" s="33"/>
     </row>
-    <row r="51" spans="1:7" ns3:dyDescent="0.2">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51" s="33"/>
       <c r="B51" s="33"/>
       <c r="C51" s="33"/>
@@ -2356,7 +2261,7 @@
       <c r="F51" s="36"/>
       <c r="G51" s="33"/>
     </row>
-    <row r="52" spans="1:7" ns3:dyDescent="0.2">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" s="33"/>
       <c r="B52" s="33"/>
       <c r="C52" s="33"/>
@@ -2365,7 +2270,7 @@
       <c r="F52" s="36"/>
       <c r="G52" s="33"/>
     </row>
-    <row r="53" spans="1:7" ht="15.75" ns3:dyDescent="0.2">
+    <row r="53" spans="1:7" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A53" s="20" t="s">
         <v>31</v>
       </c>
@@ -2381,607 +2286,607 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:7" ns3:dyDescent="0.2">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B54" s="10"/>
     </row>
-    <row r="55" spans="1:7" ns3:dyDescent="0.2">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B55" s="10"/>
     </row>
-    <row r="56" spans="1:7" ns3:dyDescent="0.2">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B56" s="10"/>
     </row>
-    <row r="57" spans="1:7" ns3:dyDescent="0.2">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B57" s="10"/>
     </row>
-    <row r="58" spans="1:7" ns3:dyDescent="0.2">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B58" s="10"/>
     </row>
-    <row r="59" spans="1:7" ns3:dyDescent="0.2">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B59" s="10"/>
     </row>
-    <row r="60" spans="1:7" ns3:dyDescent="0.2">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B60" s="10"/>
     </row>
-    <row r="61" spans="1:7" ns3:dyDescent="0.2">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B61" s="10"/>
     </row>
-    <row r="62" spans="1:7" ns3:dyDescent="0.2">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B62" s="10"/>
     </row>
-    <row r="63" spans="1:7" ns3:dyDescent="0.2">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B63" s="10"/>
     </row>
-    <row r="64" spans="1:7" ns3:dyDescent="0.2">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B64" s="10"/>
     </row>
-    <row r="65" spans="2:2" ns3:dyDescent="0.2">
+    <row r="65" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B65" s="10"/>
     </row>
-    <row r="66" spans="2:2" ns3:dyDescent="0.2">
+    <row r="66" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B66" s="10"/>
     </row>
-    <row r="67" spans="2:2" ns3:dyDescent="0.2">
+    <row r="67" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B67" s="10"/>
     </row>
-    <row r="68" spans="2:2" ns3:dyDescent="0.2">
+    <row r="68" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B68" s="10"/>
     </row>
-    <row r="69" spans="2:2" ns3:dyDescent="0.2">
+    <row r="69" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B69" s="10"/>
     </row>
-    <row r="70" spans="2:2" ns3:dyDescent="0.2">
+    <row r="70" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B70" s="10"/>
     </row>
-    <row r="71" spans="2:2" ns3:dyDescent="0.2">
+    <row r="71" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B71" s="10"/>
     </row>
-    <row r="72" spans="2:2" ns3:dyDescent="0.2">
+    <row r="72" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B72" s="10"/>
     </row>
-    <row r="73" spans="2:2" ns3:dyDescent="0.2">
+    <row r="73" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B73" s="10"/>
     </row>
-    <row r="74" spans="2:2" ns3:dyDescent="0.2">
+    <row r="74" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B74" s="10"/>
     </row>
-    <row r="75" spans="2:2" ns3:dyDescent="0.2">
+    <row r="75" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B75" s="10"/>
     </row>
-    <row r="76" spans="2:2" ht="12" customHeight="1" ns3:dyDescent="0.2">
+    <row r="76" spans="2:2" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B76" s="10"/>
     </row>
-    <row r="77" spans="2:2" ns3:dyDescent="0.2">
+    <row r="77" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B77" s="10"/>
     </row>
-    <row r="78" spans="2:2" ns3:dyDescent="0.2">
+    <row r="78" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B78" s="10"/>
     </row>
-    <row r="79" spans="2:2" ns3:dyDescent="0.2">
+    <row r="79" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B79" s="10"/>
     </row>
-    <row r="80" spans="2:2" ns3:dyDescent="0.2">
+    <row r="80" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B80" s="10"/>
     </row>
-    <row r="81" spans="2:2" ns3:dyDescent="0.2">
+    <row r="81" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B81" s="10"/>
     </row>
-    <row r="82" spans="2:2" ns3:dyDescent="0.2">
+    <row r="82" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B82" s="10"/>
     </row>
-    <row r="83" spans="2:2" ns3:dyDescent="0.2">
+    <row r="83" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B83" s="10"/>
     </row>
-    <row r="84" spans="2:2" ns3:dyDescent="0.2">
+    <row r="84" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B84" s="10"/>
     </row>
-    <row r="85" spans="2:2" ns3:dyDescent="0.2">
+    <row r="85" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B85" s="10"/>
     </row>
-    <row r="86" spans="2:2" ns3:dyDescent="0.2">
+    <row r="86" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B86" s="10"/>
     </row>
-    <row r="87" spans="2:2" ns3:dyDescent="0.2">
+    <row r="87" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B87" s="10"/>
     </row>
-    <row r="88" spans="2:2" ns3:dyDescent="0.2">
+    <row r="88" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B88" s="10"/>
     </row>
-    <row r="89" spans="2:2" ns3:dyDescent="0.2">
+    <row r="89" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B89" s="10"/>
     </row>
-    <row r="90" spans="2:2" ns3:dyDescent="0.2">
+    <row r="90" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B90" s="10"/>
     </row>
-    <row r="91" spans="2:2" ns3:dyDescent="0.2">
+    <row r="91" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B91" s="10"/>
     </row>
-    <row r="92" spans="2:2" ns3:dyDescent="0.2">
+    <row r="92" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B92" s="10"/>
     </row>
-    <row r="93" spans="2:2" ns3:dyDescent="0.2">
+    <row r="93" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B93" s="10"/>
     </row>
-    <row r="94" spans="2:2" ns3:dyDescent="0.2">
+    <row r="94" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B94" s="10"/>
     </row>
-    <row r="95" spans="2:2" ns3:dyDescent="0.2">
+    <row r="95" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B95" s="10"/>
     </row>
-    <row r="96" spans="2:2" ns3:dyDescent="0.2">
+    <row r="96" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B96" s="10"/>
     </row>
-    <row r="97" spans="2:2" ns3:dyDescent="0.2">
+    <row r="97" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B97" s="10"/>
     </row>
-    <row r="98" spans="2:2" ns3:dyDescent="0.2">
+    <row r="98" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B98" s="10"/>
     </row>
-    <row r="99" spans="2:2" ns3:dyDescent="0.2">
+    <row r="99" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B99" s="10"/>
     </row>
-    <row r="100" spans="2:2" ns3:dyDescent="0.2">
+    <row r="100" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B100" s="10"/>
     </row>
-    <row r="101" spans="2:2" ns3:dyDescent="0.2">
+    <row r="101" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B101" s="10"/>
     </row>
-    <row r="102" spans="2:2" ns3:dyDescent="0.2">
+    <row r="102" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B102" s="10"/>
     </row>
-    <row r="103" spans="2:2" ns3:dyDescent="0.2">
+    <row r="103" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B103" s="10"/>
     </row>
-    <row r="104" spans="2:2" ns3:dyDescent="0.2">
+    <row r="104" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B104" s="10"/>
     </row>
-    <row r="105" spans="2:2" ns3:dyDescent="0.2">
+    <row r="105" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B105" s="10"/>
     </row>
-    <row r="106" spans="2:2" ns3:dyDescent="0.2">
+    <row r="106" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B106" s="10"/>
     </row>
-    <row r="107" spans="2:2" ns3:dyDescent="0.2">
+    <row r="107" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B107" s="10"/>
     </row>
-    <row r="108" spans="2:2" ns3:dyDescent="0.2">
+    <row r="108" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B108" s="10"/>
     </row>
-    <row r="109" spans="2:2" ns3:dyDescent="0.2">
+    <row r="109" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B109" s="10"/>
     </row>
-    <row r="110" spans="2:2" ns3:dyDescent="0.2">
+    <row r="110" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B110" s="10"/>
     </row>
-    <row r="111" spans="2:2" ns3:dyDescent="0.2">
+    <row r="111" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B111" s="10"/>
     </row>
-    <row r="112" spans="2:2" ns3:dyDescent="0.2">
+    <row r="112" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B112" s="10"/>
     </row>
-    <row r="113" spans="2:2" ns3:dyDescent="0.2">
+    <row r="113" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B113" s="10"/>
     </row>
-    <row r="114" spans="2:2" ns3:dyDescent="0.2">
+    <row r="114" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B114" s="10"/>
     </row>
-    <row r="115" spans="2:2" ns3:dyDescent="0.2">
+    <row r="115" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B115" s="10"/>
     </row>
-    <row r="116" spans="2:2" ns3:dyDescent="0.2">
+    <row r="116" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B116" s="10"/>
     </row>
-    <row r="117" spans="2:2" ns3:dyDescent="0.2">
+    <row r="117" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B117" s="10"/>
     </row>
-    <row r="118" spans="2:2" ns3:dyDescent="0.2">
+    <row r="118" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B118" s="10"/>
     </row>
-    <row r="119" spans="2:2" ns3:dyDescent="0.2">
+    <row r="119" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B119" s="10"/>
     </row>
-    <row r="120" spans="2:2" ns3:dyDescent="0.2">
+    <row r="120" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B120" s="10"/>
     </row>
-    <row r="121" spans="2:2" ns3:dyDescent="0.2">
+    <row r="121" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B121" s="10"/>
     </row>
-    <row r="122" spans="2:2" ns3:dyDescent="0.2">
+    <row r="122" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B122" s="10"/>
     </row>
-    <row r="123" spans="2:2" ns3:dyDescent="0.2">
+    <row r="123" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B123" s="10"/>
     </row>
-    <row r="124" spans="2:2" ns3:dyDescent="0.2">
+    <row r="124" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B124" s="10"/>
     </row>
-    <row r="125" spans="2:2" ns3:dyDescent="0.2">
+    <row r="125" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B125" s="10"/>
     </row>
-    <row r="126" spans="2:2" ns3:dyDescent="0.2">
+    <row r="126" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B126" s="10"/>
     </row>
-    <row r="127" spans="2:2" ns3:dyDescent="0.2">
+    <row r="127" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B127" s="10"/>
     </row>
-    <row r="128" spans="2:2" ns3:dyDescent="0.2">
+    <row r="128" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B128" s="10"/>
     </row>
-    <row r="129" spans="2:2" ns3:dyDescent="0.2">
+    <row r="129" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B129" s="10"/>
     </row>
-    <row r="130" spans="2:2" ns3:dyDescent="0.2">
+    <row r="130" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B130" s="10"/>
     </row>
-    <row r="131" spans="2:2" ns3:dyDescent="0.2">
+    <row r="131" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B131" s="10"/>
     </row>
-    <row r="132" spans="2:2" ns3:dyDescent="0.2">
+    <row r="132" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B132" s="10"/>
     </row>
-    <row r="133" spans="2:2" ns3:dyDescent="0.2">
+    <row r="133" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B133" s="10"/>
     </row>
-    <row r="134" spans="2:2" ns3:dyDescent="0.2">
+    <row r="134" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B134" s="10"/>
     </row>
-    <row r="135" spans="2:2" ns3:dyDescent="0.2">
+    <row r="135" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B135" s="10"/>
     </row>
-    <row r="136" spans="2:2" ns3:dyDescent="0.2">
+    <row r="136" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B136" s="10"/>
     </row>
-    <row r="137" spans="2:2" ns3:dyDescent="0.2">
+    <row r="137" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B137" s="10"/>
     </row>
-    <row r="138" spans="2:2" ns3:dyDescent="0.2">
+    <row r="138" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B138" s="10"/>
     </row>
-    <row r="139" spans="2:2" ns3:dyDescent="0.2">
+    <row r="139" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B139" s="10"/>
     </row>
-    <row r="140" spans="2:2" ns3:dyDescent="0.2">
+    <row r="140" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B140" s="10"/>
     </row>
-    <row r="141" spans="2:2" ns3:dyDescent="0.2">
+    <row r="141" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B141" s="10"/>
     </row>
-    <row r="142" spans="2:2" ns3:dyDescent="0.2">
+    <row r="142" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B142" s="10"/>
     </row>
-    <row r="143" spans="2:2" ns3:dyDescent="0.2">
+    <row r="143" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B143" s="10"/>
     </row>
-    <row r="144" spans="2:2" ns3:dyDescent="0.2">
+    <row r="144" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B144" s="10"/>
     </row>
-    <row r="145" spans="2:2" ns3:dyDescent="0.2">
+    <row r="145" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B145" s="10"/>
     </row>
-    <row r="146" spans="2:2" ns3:dyDescent="0.2">
+    <row r="146" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B146" s="10"/>
     </row>
-    <row r="147" spans="2:2" ns3:dyDescent="0.2">
+    <row r="147" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B147" s="10"/>
     </row>
-    <row r="148" spans="2:2" ns3:dyDescent="0.2">
+    <row r="148" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B148" s="10"/>
     </row>
-    <row r="149" spans="2:2" ns3:dyDescent="0.2">
+    <row r="149" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B149" s="10"/>
     </row>
-    <row r="150" spans="2:2" ns3:dyDescent="0.2">
+    <row r="150" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B150" s="10"/>
     </row>
-    <row r="151" spans="2:2" ns3:dyDescent="0.2">
+    <row r="151" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B151" s="10"/>
     </row>
-    <row r="152" spans="2:2" ns3:dyDescent="0.2">
+    <row r="152" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B152" s="10"/>
     </row>
-    <row r="153" spans="2:2" ns3:dyDescent="0.2">
+    <row r="153" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B153" s="10"/>
     </row>
-    <row r="154" spans="2:2" ns3:dyDescent="0.2">
+    <row r="154" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B154" s="10"/>
     </row>
-    <row r="155" spans="2:2" ns3:dyDescent="0.2">
+    <row r="155" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B155" s="10"/>
     </row>
-    <row r="156" spans="2:2" ns3:dyDescent="0.2">
+    <row r="156" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B156" s="10"/>
     </row>
-    <row r="157" spans="2:2" ns3:dyDescent="0.2">
+    <row r="157" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B157" s="10"/>
     </row>
-    <row r="158" spans="2:2" ns3:dyDescent="0.2">
+    <row r="158" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B158" s="10"/>
     </row>
-    <row r="159" spans="2:2" ns3:dyDescent="0.2">
+    <row r="159" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B159" s="10"/>
     </row>
-    <row r="160" spans="2:2" ns3:dyDescent="0.2">
+    <row r="160" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B160" s="10"/>
     </row>
-    <row r="161" spans="2:2" ns3:dyDescent="0.2">
+    <row r="161" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B161" s="10"/>
     </row>
-    <row r="162" spans="2:2" ns3:dyDescent="0.2">
+    <row r="162" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B162" s="10"/>
     </row>
-    <row r="163" spans="2:2" ns3:dyDescent="0.2">
+    <row r="163" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B163" s="10"/>
     </row>
-    <row r="164" spans="2:2" ns3:dyDescent="0.2">
+    <row r="164" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B164" s="10"/>
     </row>
-    <row r="165" spans="2:2" ns3:dyDescent="0.2">
+    <row r="165" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B165" s="10"/>
     </row>
-    <row r="166" spans="2:2" ns3:dyDescent="0.2">
+    <row r="166" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B166" s="10"/>
     </row>
-    <row r="167" spans="2:2" ns3:dyDescent="0.2">
+    <row r="167" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B167" s="10"/>
     </row>
-    <row r="168" spans="2:2" ns3:dyDescent="0.2">
+    <row r="168" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B168" s="10"/>
     </row>
-    <row r="169" spans="2:2" ns3:dyDescent="0.2">
+    <row r="169" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B169" s="10"/>
     </row>
-    <row r="170" spans="2:2" ns3:dyDescent="0.2">
+    <row r="170" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B170" s="10"/>
     </row>
-    <row r="171" spans="2:2" ns3:dyDescent="0.2">
+    <row r="171" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B171" s="10"/>
     </row>
-    <row r="172" spans="2:2" ns3:dyDescent="0.2">
+    <row r="172" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B172" s="10"/>
     </row>
-    <row r="173" spans="2:2" ns3:dyDescent="0.2">
+    <row r="173" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B173" s="10"/>
     </row>
-    <row r="174" spans="2:2" ns3:dyDescent="0.2">
+    <row r="174" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B174" s="10"/>
     </row>
-    <row r="175" spans="2:2" ns3:dyDescent="0.2">
+    <row r="175" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B175" s="10"/>
     </row>
-    <row r="176" spans="2:2" ns3:dyDescent="0.2">
+    <row r="176" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B176" s="10"/>
     </row>
-    <row r="177" spans="2:2" ns3:dyDescent="0.2">
+    <row r="177" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B177" s="10"/>
     </row>
-    <row r="178" spans="2:2" ns3:dyDescent="0.2">
+    <row r="178" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B178" s="10"/>
     </row>
-    <row r="179" spans="2:2" ns3:dyDescent="0.2">
+    <row r="179" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B179" s="10"/>
     </row>
-    <row r="180" spans="2:2" ns3:dyDescent="0.2">
+    <row r="180" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B180" s="10"/>
     </row>
-    <row r="181" spans="2:2" ns3:dyDescent="0.2">
+    <row r="181" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B181" s="10"/>
     </row>
-    <row r="182" spans="2:2" ns3:dyDescent="0.2">
+    <row r="182" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B182" s="10"/>
     </row>
-    <row r="183" spans="2:2" ns3:dyDescent="0.2">
+    <row r="183" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B183" s="10"/>
     </row>
-    <row r="184" spans="2:2" ns3:dyDescent="0.2">
+    <row r="184" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B184" s="10"/>
     </row>
-    <row r="185" spans="2:2" ns3:dyDescent="0.2">
+    <row r="185" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B185" s="10"/>
     </row>
-    <row r="186" spans="2:2" ns3:dyDescent="0.2">
+    <row r="186" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B186" s="10"/>
     </row>
-    <row r="187" spans="2:2" ns3:dyDescent="0.2">
+    <row r="187" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B187" s="10"/>
     </row>
-    <row r="188" spans="2:2" ns3:dyDescent="0.2">
+    <row r="188" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B188" s="10"/>
     </row>
-    <row r="189" spans="2:2" ns3:dyDescent="0.2">
+    <row r="189" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B189" s="10"/>
     </row>
-    <row r="190" spans="2:2" ns3:dyDescent="0.2">
+    <row r="190" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B190" s="10"/>
     </row>
-    <row r="191" spans="2:2" ns3:dyDescent="0.2">
+    <row r="191" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B191" s="10"/>
     </row>
-    <row r="192" spans="2:2" ns3:dyDescent="0.2">
+    <row r="192" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B192" s="10"/>
     </row>
-    <row r="193" spans="2:2" ns3:dyDescent="0.2">
+    <row r="193" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B193" s="10"/>
     </row>
-    <row r="194" spans="2:2" ns3:dyDescent="0.2">
+    <row r="194" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B194" s="10"/>
     </row>
-    <row r="195" spans="2:2" ns3:dyDescent="0.2">
+    <row r="195" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B195" s="10"/>
     </row>
-    <row r="196" spans="2:2" ns3:dyDescent="0.2">
+    <row r="196" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B196" s="10"/>
     </row>
-    <row r="197" spans="2:2" ns3:dyDescent="0.2">
+    <row r="197" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B197" s="10"/>
     </row>
-    <row r="198" spans="2:2" ns3:dyDescent="0.2">
+    <row r="198" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B198" s="10"/>
     </row>
-    <row r="199" spans="2:2" ns3:dyDescent="0.2">
+    <row r="199" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B199" s="10"/>
     </row>
-    <row r="200" spans="2:2" ns3:dyDescent="0.2">
+    <row r="200" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B200" s="10"/>
     </row>
-    <row r="201" spans="2:2" ns3:dyDescent="0.2">
+    <row r="201" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B201" s="10"/>
     </row>
-    <row r="202" spans="2:2" ns3:dyDescent="0.2">
+    <row r="202" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B202" s="10"/>
     </row>
-    <row r="203" spans="2:2" ns3:dyDescent="0.2">
+    <row r="203" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B203" s="10"/>
     </row>
-    <row r="204" spans="2:2" ns3:dyDescent="0.2">
+    <row r="204" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B204" s="10"/>
     </row>
-    <row r="205" spans="2:2" ns3:dyDescent="0.2">
+    <row r="205" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B205" s="10"/>
     </row>
-    <row r="206" spans="2:2" ns3:dyDescent="0.2">
+    <row r="206" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B206" s="10"/>
     </row>
-    <row r="207" spans="2:2" ns3:dyDescent="0.2">
+    <row r="207" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B207" s="10"/>
     </row>
-    <row r="208" spans="2:2" ns3:dyDescent="0.2">
+    <row r="208" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B208" s="10"/>
     </row>
-    <row r="209" spans="2:2" ns3:dyDescent="0.2">
+    <row r="209" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B209" s="10"/>
     </row>
-    <row r="210" spans="2:2" ns3:dyDescent="0.2">
+    <row r="210" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B210" s="10"/>
     </row>
-    <row r="211" spans="2:2" ns3:dyDescent="0.2">
+    <row r="211" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B211" s="10"/>
     </row>
-    <row r="212" spans="2:2" ns3:dyDescent="0.2">
+    <row r="212" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B212" s="10"/>
     </row>
-    <row r="213" spans="2:2" ns3:dyDescent="0.2">
+    <row r="213" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B213" s="10"/>
     </row>
-    <row r="214" spans="2:2" ns3:dyDescent="0.2">
+    <row r="214" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B214" s="10"/>
     </row>
-    <row r="215" spans="2:2" ns3:dyDescent="0.2">
+    <row r="215" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B215" s="10"/>
     </row>
-    <row r="216" spans="2:2" ns3:dyDescent="0.2">
+    <row r="216" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B216" s="10"/>
     </row>
-    <row r="217" spans="2:2" ns3:dyDescent="0.2">
+    <row r="217" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B217" s="10"/>
     </row>
-    <row r="218" spans="2:2" ns3:dyDescent="0.2">
+    <row r="218" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B218" s="10"/>
     </row>
-    <row r="219" spans="2:2" ns3:dyDescent="0.2">
+    <row r="219" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B219" s="10"/>
     </row>
-    <row r="220" spans="2:2" ns3:dyDescent="0.2">
+    <row r="220" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B220" s="10"/>
     </row>
-    <row r="221" spans="2:2" ns3:dyDescent="0.2">
+    <row r="221" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B221" s="10"/>
     </row>
-    <row r="222" spans="2:2" ns3:dyDescent="0.2">
+    <row r="222" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B222" s="10"/>
     </row>
-    <row r="223" spans="2:2" ns3:dyDescent="0.2">
+    <row r="223" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B223" s="10"/>
     </row>
-    <row r="224" spans="2:2" ns3:dyDescent="0.2">
+    <row r="224" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B224" s="10"/>
     </row>
-    <row r="225" spans="2:2" ns3:dyDescent="0.2">
+    <row r="225" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B225" s="10"/>
     </row>
-    <row r="226" spans="2:2" ns3:dyDescent="0.2">
+    <row r="226" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B226" s="10"/>
     </row>
-    <row r="227" spans="2:2" ns3:dyDescent="0.2">
+    <row r="227" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B227" s="10"/>
     </row>
-    <row r="228" spans="2:2" ns3:dyDescent="0.2">
+    <row r="228" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B228" s="10"/>
     </row>
-    <row r="229" spans="2:2" ns3:dyDescent="0.2">
+    <row r="229" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B229" s="10"/>
     </row>
-    <row r="230" spans="2:2" ns3:dyDescent="0.2">
+    <row r="230" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B230" s="10"/>
     </row>
-    <row r="231" spans="2:2" ns3:dyDescent="0.2">
+    <row r="231" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B231" s="10"/>
     </row>
-    <row r="232" spans="2:2" ns3:dyDescent="0.2">
+    <row r="232" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B232" s="10"/>
     </row>
-    <row r="233" spans="2:2" ns3:dyDescent="0.2">
+    <row r="233" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B233" s="10"/>
     </row>
-    <row r="234" spans="2:2" ns3:dyDescent="0.2">
+    <row r="234" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B234" s="10"/>
     </row>
-    <row r="235" spans="2:2" ns3:dyDescent="0.2">
+    <row r="235" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B235" s="10"/>
     </row>
-    <row r="236" spans="2:2" ns3:dyDescent="0.2">
+    <row r="236" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B236" s="10"/>
     </row>
-    <row r="237" spans="2:2" ns3:dyDescent="0.2">
+    <row r="237" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B237" s="10"/>
     </row>
-    <row r="238" spans="2:2" ns3:dyDescent="0.2">
+    <row r="238" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B238" s="10"/>
     </row>
-    <row r="239" spans="2:2" ns3:dyDescent="0.2">
+    <row r="239" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B239" s="10"/>
     </row>
-    <row r="240" spans="2:2" ns3:dyDescent="0.2">
+    <row r="240" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B240" s="10"/>
     </row>
-    <row r="241" spans="2:2" ns3:dyDescent="0.2">
+    <row r="241" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B241" s="10"/>
     </row>
-    <row r="242" spans="2:2" ns3:dyDescent="0.2">
+    <row r="242" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B242" s="10"/>
     </row>
-    <row r="243" spans="2:2" ns3:dyDescent="0.2">
+    <row r="243" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B243" s="10"/>
     </row>
-    <row r="244" spans="2:2" ns3:dyDescent="0.2">
+    <row r="244" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B244" s="10"/>
     </row>
-    <row r="245" spans="2:2" ns3:dyDescent="0.2">
+    <row r="245" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B245" s="10"/>
     </row>
-    <row r="246" spans="2:2" ns3:dyDescent="0.2">
+    <row r="246" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B246" s="10"/>
     </row>
-    <row r="247" spans="2:2" ns3:dyDescent="0.2">
+    <row r="247" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B247" s="10"/>
     </row>
-    <row r="248" spans="2:2" ns3:dyDescent="0.2">
+    <row r="248" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B248" s="10"/>
     </row>
-    <row r="249" spans="2:2" ns3:dyDescent="0.2">
+    <row r="249" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B249" s="10"/>
     </row>
-    <row r="250" spans="2:2" ns3:dyDescent="0.2">
+    <row r="250" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B250" s="10"/>
     </row>
-    <row r="251" spans="2:2" ns3:dyDescent="0.2">
+    <row r="251" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B251" s="10"/>
     </row>
-    <row r="252" spans="2:2" ns3:dyDescent="0.2">
+    <row r="252" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B252" s="10"/>
     </row>
-    <row r="253" spans="2:2" ns3:dyDescent="0.2">
+    <row r="253" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B253" s="10"/>
     </row>
-    <row r="254" spans="2:2" ns3:dyDescent="0.2">
+    <row r="254" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B254" s="10"/>
     </row>
   </sheetData>
@@ -2998,100 +2903,100 @@
   <headerFooter alignWithMargins="0"/>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>
-  <ns1:AlternateContent>
-    <ns1:Choice Requires="x14">
+  <mc:AlternateContent>
+    <mc:Choice Requires="x14">
       <controls>
-        <ns1:AlternateContent>
-          <ns1:Choice Requires="x14">
+        <mc:AlternateContent>
+          <mc:Choice Requires="x14">
             <control shapeId="1025" r:id="rId4" name="Check Box 1">
               <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
                 <anchor moveWithCells="1">
                   <from>
-                    <ns5:col>1</ns5:col>
-                    <ns5:colOff>0</ns5:colOff>
-                    <ns5:row>8</ns5:row>
-                    <ns5:rowOff>9525</ns5:rowOff>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>0</xdr:colOff>
+                    <xdr:row>8</xdr:row>
+                    <xdr:rowOff>9525</xdr:rowOff>
                   </from>
                   <to>
-                    <ns5:col>1</ns5:col>
-                    <ns5:colOff>895350</ns5:colOff>
-                    <ns5:row>9</ns5:row>
-                    <ns5:rowOff>95250</ns5:rowOff>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>895350</xdr:colOff>
+                    <xdr:row>9</xdr:row>
+                    <xdr:rowOff>95250</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
             </control>
-          </ns1:Choice>
-        </ns1:AlternateContent>
-        <ns1:AlternateContent>
-          <ns1:Choice Requires="x14">
+          </mc:Choice>
+        </mc:AlternateContent>
+        <mc:AlternateContent>
+          <mc:Choice Requires="x14">
             <control shapeId="1030" r:id="rId5" name="Check Box 6">
               <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
                 <anchor moveWithCells="1">
                   <from>
-                    <ns5:col>1</ns5:col>
-                    <ns5:colOff>0</ns5:colOff>
-                    <ns5:row>5</ns5:row>
-                    <ns5:rowOff>0</ns5:rowOff>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>0</xdr:colOff>
+                    <xdr:row>5</xdr:row>
+                    <xdr:rowOff>0</xdr:rowOff>
                   </from>
                   <to>
-                    <ns5:col>1</ns5:col>
-                    <ns5:colOff>685800</ns5:colOff>
-                    <ns5:row>5</ns5:row>
-                    <ns5:rowOff>219075</ns5:rowOff>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>685800</xdr:colOff>
+                    <xdr:row>5</xdr:row>
+                    <xdr:rowOff>219075</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
             </control>
-          </ns1:Choice>
-        </ns1:AlternateContent>
-        <ns1:AlternateContent>
-          <ns1:Choice Requires="x14">
+          </mc:Choice>
+        </mc:AlternateContent>
+        <mc:AlternateContent>
+          <mc:Choice Requires="x14">
             <control shapeId="1031" r:id="rId6" name="Check Box 7">
               <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
                 <anchor moveWithCells="1">
                   <from>
-                    <ns5:col>1</ns5:col>
-                    <ns5:colOff>0</ns5:colOff>
-                    <ns5:row>6</ns5:row>
-                    <ns5:rowOff>0</ns5:rowOff>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>0</xdr:colOff>
+                    <xdr:row>6</xdr:row>
+                    <xdr:rowOff>0</xdr:rowOff>
                   </from>
                   <to>
-                    <ns5:col>1</ns5:col>
-                    <ns5:colOff>685800</ns5:colOff>
-                    <ns5:row>7</ns5:row>
-                    <ns5:rowOff>0</ns5:rowOff>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>685800</xdr:colOff>
+                    <xdr:row>7</xdr:row>
+                    <xdr:rowOff>0</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
             </control>
-          </ns1:Choice>
-        </ns1:AlternateContent>
-        <ns1:AlternateContent>
-          <ns1:Choice Requires="x14">
+          </mc:Choice>
+        </mc:AlternateContent>
+        <mc:AlternateContent>
+          <mc:Choice Requires="x14">
             <control shapeId="1032" r:id="rId7" name="Check Box 8">
               <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
                 <anchor moveWithCells="1">
                   <from>
-                    <ns5:col>1</ns5:col>
-                    <ns5:colOff>0</ns5:colOff>
-                    <ns5:row>9</ns5:row>
-                    <ns5:rowOff>9525</ns5:rowOff>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>0</xdr:colOff>
+                    <xdr:row>9</xdr:row>
+                    <xdr:rowOff>9525</xdr:rowOff>
                   </from>
                   <to>
-                    <ns5:col>1</ns5:col>
-                    <ns5:colOff>685800</ns5:colOff>
-                    <ns5:row>10</ns5:row>
-                    <ns5:rowOff>66675</ns5:rowOff>
+                    <xdr:col>1</xdr:col>
+                    <xdr:colOff>685800</xdr:colOff>
+                    <xdr:row>10</xdr:row>
+                    <xdr:rowOff>66675</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
             </control>
-          </ns1:Choice>
-        </ns1:AlternateContent>
+          </mc:Choice>
+        </mc:AlternateContent>
       </controls>
-    </ns1:Choice>
-  </ns1:AlternateContent>
+    </mc:Choice>
+  </mc:AlternateContent>
 </worksheet>
 </file>
 

</xml_diff>